<commit_message>
Search precision and image search: suggest only documents that really match
- Evidence rule: a document is suggested only if it contains at least one query keyword (or related term) or a
  passage is genuinely relevant in meaning (semantic ranker >= 2.0, or cosine >= 0.45 without the ranker).
  Unrelated documents that vector search always returns, scored about 1-2 by the ranker (25-50%), are hidden.
  Thresholds in Config/search.yaml; the API reports matchedTerms and hiddenNoEvidence.
- Precision filters: minimum match 30%, relative cutoff (60% of the best match), exact-phrase bonus, queries
  naming a code, file name, figure label or quoted phrase only match documents containing it; no padding.
- Image search: images extracted from PDF, Word and Excel are indexed with captions and shown with results.
- Docs and tests updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/sample_docs/Cloud-Migration-Project-Plan.xlsx
+++ b/Data/sample_docs/Cloud-Migration-Project-Plan.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -137,6 +138,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6096000" cy="2857500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -940,4 +971,43 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Target architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Figure 1: Target cloud architecture diagram (landing zone, hub network, billing and meter data platforms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Both platforms run behind the hub network firewall and reach the old data centre over ExpressRoute.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>